<commit_message>
reports update with earmarked data excluded
</commit_message>
<xml_diff>
--- a/reports/pro-crypto/pro-crypto-independent-expenditure-region.xlsx
+++ b/reports/pro-crypto/pro-crypto-independent-expenditure-region.xlsx
@@ -42,6 +42,63 @@
     <x:t>expenditure_description</x:t>
   </x:si>
   <x:si>
+    <x:t>C00915181</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FELLOWSHIP PAC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FULLER, CLAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUPPORT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOORE, FELIX BARRY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>COLLINS, MICHAEL A JR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MORRIS, NATE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIGUEZ, BLAKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LETLOW, JULIA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RICKETTS, PETE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAXTON, WARREN KENNETH JR.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TX</x:t>
+  </x:si>
+  <x:si>
     <x:t>C00835959</x:t>
   </x:si>
   <x:si>
@@ -69,9 +126,6 @@
     <x:t>STRATTON, JULIANA</x:t>
   </x:si>
   <x:si>
-    <x:t>00</x:t>
-  </x:si>
-  <x:si>
     <x:t>C00836221</x:t>
   </x:si>
   <x:si>
@@ -84,15 +138,9 @@
     <x:t>AR</x:t>
   </x:si>
   <x:si>
-    <x:t>SUPPORT</x:t>
-  </x:si>
-  <x:si>
     <x:t>MOORE, TIM</x:t>
   </x:si>
   <x:si>
-    <x:t>14</x:t>
-  </x:si>
-  <x:si>
     <x:t>NC</x:t>
   </x:si>
   <x:si>
@@ -117,9 +165,6 @@
     <x:t>08</x:t>
   </x:si>
   <x:si>
-    <x:t>TX</x:t>
-  </x:si>
-  <x:si>
     <x:t>GOBER, CHRIS</x:t>
   </x:si>
   <x:si>
@@ -132,12 +177,6 @@
     <x:t>22</x:t>
   </x:si>
   <x:si>
-    <x:t>MOORE, FELIX BARRY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AL</x:t>
-  </x:si>
-  <x:si>
     <x:t>C00848440</x:t>
   </x:si>
   <x:si>
@@ -186,9 +225,6 @@
     <x:t>SCOTT, DAVID ALBERT</x:t>
   </x:si>
   <x:si>
-    <x:t>GA</x:t>
-  </x:si>
-  <x:si>
     <x:t>CLARK, JASMINE</x:t>
   </x:si>
   <x:si>
@@ -199,42 +235,6 @@
   </x:si>
   <x:si>
     <x:t>KRISHNAMOORTHI, S</x:t>
-  </x:si>
-  <x:si>
-    <x:t>C00915181</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FELLOWSHIP PAC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FULLER, CLAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>COLLINS, MICHAEL A JR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MORRIS, NATE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIGUEZ, BLAKE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LETLOW, JULIA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RICKETTS, PETE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAXTON, WARREN KENNETH JR.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -723,7 +723,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="1">
-        <x:v>817066</x:v>
+        <x:v>300000</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
         <x:v>12</x:v>
@@ -743,10 +743,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="1">
-        <x:v>1803694</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="G3" s="1" t="s">
         <x:v>12</x:v>
@@ -760,16 +760,16 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F4" s="1">
-        <x:v>5168736</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="G4" s="1" t="s">
         <x:v>12</x:v>
@@ -777,298 +777,298 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B5" s="1" t="s">
+      <x:c r="D5" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="C5" s="1" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D5" s="1" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E5" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="F5" s="1">
-        <x:v>418058</x:v>
+        <x:v>850000</x:v>
       </x:c>
       <x:c r="G5" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="A6" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F6" s="1">
-        <x:v>80948</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="G6" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
       <x:c r="A7" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F7" s="1">
-        <x:v>558813</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="G7" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>29</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F8" s="1">
-        <x:v>1673736</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="G8" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F9" s="1">
-        <x:v>771658</x:v>
+        <x:v>1750000</x:v>
       </x:c>
       <x:c r="G9" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F10" s="1">
-        <x:v>91656</x:v>
+        <x:v>817066</x:v>
       </x:c>
       <x:c r="G10" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:7">
       <x:c r="A11" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F11" s="1">
-        <x:v>141263</x:v>
+        <x:v>1803694</x:v>
       </x:c>
       <x:c r="G11" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F12" s="1">
-        <x:v>5017853</x:v>
+        <x:v>5168736</x:v>
       </x:c>
       <x:c r="G12" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="A13" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F13" s="1">
-        <x:v>83860</x:v>
+        <x:v>418058</x:v>
       </x:c>
       <x:c r="G13" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:7">
       <x:c r="A14" s="1" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B14" s="1" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="s">
+      <x:c r="D14" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C14" s="1" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D14" s="1" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="E14" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="F14" s="1">
-        <x:v>515519</x:v>
+        <x:v>80948</x:v>
       </x:c>
       <x:c r="G14" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="A15" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F15" s="1">
-        <x:v>1564215</x:v>
+        <x:v>558813</x:v>
       </x:c>
       <x:c r="G15" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="A16" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F16" s="1">
-        <x:v>1012792</x:v>
+        <x:v>1673736</x:v>
       </x:c>
       <x:c r="G16" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:7">
       <x:c r="A17" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
         <x:v>47</x:v>
       </x:c>
       <x:c r="E17" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F17" s="1">
-        <x:v>20483</x:v>
+        <x:v>771658</x:v>
       </x:c>
       <x:c r="G17" s="1" t="s">
         <x:v>12</x:v>
@@ -1076,45 +1076,45 @@
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="A18" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E18" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F18" s="1">
-        <x:v>91847</x:v>
+        <x:v>91656</x:v>
       </x:c>
       <x:c r="G18" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="A19" s="1" t="s">
-        <x:v>7</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E19" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F19" s="1">
-        <x:v>672092</x:v>
+        <x:v>141263</x:v>
       </x:c>
       <x:c r="G19" s="1" t="s">
         <x:v>12</x:v>
@@ -1122,22 +1122,22 @@
     </x:row>
     <x:row r="20" spans="1:7">
       <x:c r="A20" s="1" t="s">
-        <x:v>7</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D20" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D20" s="1" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E20" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="F20" s="1">
-        <x:v>4697360</x:v>
+        <x:v>5017853</x:v>
       </x:c>
       <x:c r="G20" s="1" t="s">
         <x:v>12</x:v>
@@ -1145,229 +1145,229 @@
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="A21" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E21" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F21" s="1">
-        <x:v>418060</x:v>
+        <x:v>83860</x:v>
       </x:c>
       <x:c r="G21" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="A22" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E22" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F22" s="1">
-        <x:v>80948</x:v>
+        <x:v>515519</x:v>
       </x:c>
       <x:c r="G22" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:7">
       <x:c r="A23" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E23" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F23" s="1">
-        <x:v>771658</x:v>
+        <x:v>1564215</x:v>
       </x:c>
       <x:c r="G23" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="A24" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E24" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F24" s="1">
-        <x:v>91656</x:v>
+        <x:v>1012792</x:v>
       </x:c>
       <x:c r="G24" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="A25" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E25" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F25" s="1">
-        <x:v>141263</x:v>
+        <x:v>20483</x:v>
       </x:c>
       <x:c r="G25" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:7">
       <x:c r="A26" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E26" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F26" s="1">
-        <x:v>5031161</x:v>
+        <x:v>91847</x:v>
       </x:c>
       <x:c r="G26" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:7">
       <x:c r="A27" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E27" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F27" s="1">
-        <x:v>56045</x:v>
+        <x:v>672092</x:v>
       </x:c>
       <x:c r="G27" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:7">
       <x:c r="A28" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>56</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D28" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E28" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F28" s="1">
-        <x:v>2067216</x:v>
+        <x:v>4697360</x:v>
       </x:c>
       <x:c r="G28" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:7">
       <x:c r="A29" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D29" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E29" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F29" s="1">
-        <x:v>41493</x:v>
+        <x:v>418060</x:v>
       </x:c>
       <x:c r="G29" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:7">
       <x:c r="A30" s="1" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B30" s="1" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C30" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B30" s="1" t="s">
+      <x:c r="D30" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E30" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C30" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D30" s="1" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E30" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="F30" s="1">
-        <x:v>119644</x:v>
+        <x:v>80948</x:v>
       </x:c>
       <x:c r="G30" s="1" t="s">
         <x:v>12</x:v>
@@ -1375,232 +1375,232 @@
     </x:row>
     <x:row r="31" spans="1:7">
       <x:c r="A31" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C31" s="1" t="s">
-        <x:v>57</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E31" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F31" s="1">
-        <x:v>285008</x:v>
+        <x:v>771658</x:v>
       </x:c>
       <x:c r="G31" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:7">
       <x:c r="A32" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C32" s="1" t="s">
-        <x:v>59</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D32" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E32" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F32" s="1">
-        <x:v>30183</x:v>
+        <x:v>91656</x:v>
       </x:c>
       <x:c r="G32" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:7">
       <x:c r="A33" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E33" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F33" s="1">
-        <x:v>300000</x:v>
+        <x:v>141263</x:v>
       </x:c>
       <x:c r="G33" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:7">
       <x:c r="A34" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D34" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E34" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F34" s="1">
-        <x:v>350000</x:v>
+        <x:v>5031161</x:v>
       </x:c>
       <x:c r="G34" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:7">
       <x:c r="A35" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D35" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E35" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F35" s="1">
-        <x:v>350000</x:v>
+        <x:v>56045</x:v>
       </x:c>
       <x:c r="G35" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:7">
       <x:c r="A36" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E36" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F36" s="1">
-        <x:v>850000</x:v>
+        <x:v>2067216</x:v>
       </x:c>
       <x:c r="G36" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:7">
       <x:c r="A37" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E37" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F37" s="1">
-        <x:v>250000</x:v>
+        <x:v>41493</x:v>
       </x:c>
       <x:c r="G37" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:7">
       <x:c r="A38" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E38" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F38" s="1">
-        <x:v>350000</x:v>
+        <x:v>119644</x:v>
       </x:c>
       <x:c r="G38" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:7">
       <x:c r="A39" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
         <x:v>69</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E39" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F39" s="1">
-        <x:v>350000</x:v>
+        <x:v>285008</x:v>
       </x:c>
       <x:c r="G39" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:7">
       <x:c r="A40" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C40" s="1" t="s">
         <x:v>71</x:v>
       </x:c>
       <x:c r="D40" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E40" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F40" s="1">
-        <x:v>1750000</x:v>
+        <x:v>30183</x:v>
       </x:c>
       <x:c r="G40" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1649,478 +1649,478 @@
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D2" s="1">
         <x:v>10399014</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D3" s="1">
         <x:v>836118</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B4" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D4" s="1">
         <x:v>558813</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>29</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D5" s="1">
         <x:v>1673736</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D6" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D7" s="1">
         <x:v>56045</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
       <x:c r="A8" s="1" t="s">
-        <x:v>56</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D8" s="1">
         <x:v>2067216</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D9" s="1">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="1" t="s">
-        <x:v>57</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D10" s="1">
         <x:v>285008</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:5">
       <x:c r="A11" s="1" t="s">
-        <x:v>59</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D11" s="1">
         <x:v>30183</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:5">
       <x:c r="A12" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D12" s="1">
         <x:v>9985740</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:5">
       <x:c r="A13" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D13" s="1">
         <x:v>817066</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:5">
       <x:c r="A14" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D14" s="1">
         <x:v>2475786</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:5">
       <x:c r="A15" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D15" s="1">
         <x:v>557012</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:5">
       <x:c r="A16" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D16" s="1">
         <x:v>83860</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:5">
       <x:c r="A17" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D17" s="1">
         <x:v>850000</x:v>
       </x:c>
       <x:c r="E17" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:5">
       <x:c r="A18" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D18" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="E18" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:5">
       <x:c r="A19" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D19" s="1">
         <x:v>250000</x:v>
       </x:c>
       <x:c r="E19" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:5">
       <x:c r="A20" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D20" s="1">
         <x:v>91847</x:v>
       </x:c>
       <x:c r="E20" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:5">
       <x:c r="A21" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D21" s="1">
         <x:v>161896</x:v>
       </x:c>
       <x:c r="E21" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:5">
       <x:c r="A22" s="1" t="s">
-        <x:v>69</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D22" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="E22" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:5">
       <x:c r="A23" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D23" s="1">
         <x:v>1750000</x:v>
       </x:c>
       <x:c r="E23" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:5">
       <x:c r="A24" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D24" s="1">
         <x:v>1543316</x:v>
       </x:c>
       <x:c r="E24" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:5">
       <x:c r="A25" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D25" s="1">
         <x:v>183312</x:v>
       </x:c>
       <x:c r="E25" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:5">
       <x:c r="A26" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D26" s="1">
         <x:v>1564215</x:v>
       </x:c>
       <x:c r="E26" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:5">
       <x:c r="A27" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D27" s="1">
         <x:v>282526</x:v>
       </x:c>
       <x:c r="E27" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:5">
       <x:c r="A28" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D28" s="1">
         <x:v>20483</x:v>
       </x:c>
       <x:c r="E28" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:5">
       <x:c r="A29" s="1" t="s">
-        <x:v>46</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D29" s="1">
         <x:v>1012792</x:v>
       </x:c>
       <x:c r="E29" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2165,366 +2165,366 @@
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C2" s="1">
         <x:v>10399014</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C3" s="1">
         <x:v>836118</x:v>
       </x:c>
       <x:c r="D3" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
       <x:c r="A4" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B4" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C4" s="1">
         <x:v>558813</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="1" t="s">
-        <x:v>29</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C5" s="1">
         <x:v>1673736</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C6" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="1">
         <x:v>56045</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
       <x:c r="A8" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C8" s="1">
         <x:v>2067216</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C9" s="1">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:4">
       <x:c r="A10" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C10" s="1">
         <x:v>315191</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:4">
       <x:c r="A11" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C11" s="1">
         <x:v>9985740</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:4">
       <x:c r="A12" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C12" s="1">
         <x:v>817066</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:4">
       <x:c r="A13" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C13" s="1">
         <x:v>2475786</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:4">
       <x:c r="A14" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C14" s="1">
         <x:v>557012</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:4">
       <x:c r="A15" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C15" s="1">
         <x:v>83860</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:4">
       <x:c r="A16" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C16" s="1">
         <x:v>850000</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:4">
       <x:c r="A17" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C17" s="1">
         <x:v>600000</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:4">
       <x:c r="A18" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C18" s="1">
         <x:v>91847</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:4">
       <x:c r="A19" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C19" s="1">
         <x:v>161896</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:4">
       <x:c r="A20" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C20" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="D20" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:4">
       <x:c r="A21" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C21" s="1">
         <x:v>1750000</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:4">
       <x:c r="A22" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C22" s="1">
         <x:v>1543316</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:4">
       <x:c r="A23" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C23" s="1">
         <x:v>183312</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:4">
       <x:c r="A24" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C24" s="1">
         <x:v>1564215</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:4">
       <x:c r="A25" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C25" s="1">
         <x:v>282526</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:4">
       <x:c r="A26" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C26" s="1">
         <x:v>20483</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:4">
       <x:c r="A27" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C27" s="1">
         <x:v>1012792</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2565,167 +2565,167 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B2" s="1">
         <x:v>10399014</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B3" s="1">
         <x:v>836118</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B4" s="1">
         <x:v>2232549</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B5" s="1">
         <x:v>56045</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B6" s="1">
         <x:v>2717216</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B7" s="1">
         <x:v>13278592</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B8" s="1">
         <x:v>956063</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B9" s="1">
         <x:v>850000</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:3">
       <x:c r="A10" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B10" s="1">
         <x:v>600000</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:3">
       <x:c r="A11" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B11" s="1">
         <x:v>91847</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:3">
       <x:c r="A12" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B12" s="1">
         <x:v>161896</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:3">
       <x:c r="A13" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B13" s="1">
         <x:v>350000</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:3">
       <x:c r="A14" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B14" s="1">
         <x:v>5323369</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:3">
       <x:c r="A15" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B15" s="1">
         <x:v>20483</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:3">
       <x:c r="A16" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B16" s="1">
         <x:v>1012792</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2762,7 +2762,7 @@
     </x:row>
     <x:row r="2" spans="1:2">
       <x:c r="A2" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B2" s="1">
         <x:v>10399014</x:v>
@@ -2770,7 +2770,7 @@
     </x:row>
     <x:row r="3" spans="1:2">
       <x:c r="A3" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B3" s="1">
         <x:v>836118</x:v>
@@ -2778,7 +2778,7 @@
     </x:row>
     <x:row r="4" spans="1:2">
       <x:c r="A4" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B4" s="1">
         <x:v>2232549</x:v>
@@ -2786,7 +2786,7 @@
     </x:row>
     <x:row r="5" spans="1:2">
       <x:c r="A5" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B5" s="1">
         <x:v>2773261</x:v>
@@ -2794,7 +2794,7 @@
     </x:row>
     <x:row r="6" spans="1:2">
       <x:c r="A6" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B6" s="1">
         <x:v>14234655</x:v>
@@ -2802,7 +2802,7 @@
     </x:row>
     <x:row r="7" spans="1:2">
       <x:c r="A7" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B7" s="1">
         <x:v>850000</x:v>
@@ -2810,7 +2810,7 @@
     </x:row>
     <x:row r="8" spans="1:2">
       <x:c r="A8" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B8" s="1">
         <x:v>600000</x:v>
@@ -2818,7 +2818,7 @@
     </x:row>
     <x:row r="9" spans="1:2">
       <x:c r="A9" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B9" s="1">
         <x:v>91847</x:v>
@@ -2826,7 +2826,7 @@
     </x:row>
     <x:row r="10" spans="1:2">
       <x:c r="A10" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B10" s="1">
         <x:v>161896</x:v>
@@ -2834,7 +2834,7 @@
     </x:row>
     <x:row r="11" spans="1:2">
       <x:c r="A11" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B11" s="1">
         <x:v>350000</x:v>
@@ -2842,7 +2842,7 @@
     </x:row>
     <x:row r="12" spans="1:2">
       <x:c r="A12" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B12" s="1">
         <x:v>5323369</x:v>
@@ -2850,7 +2850,7 @@
     </x:row>
     <x:row r="13" spans="1:2">
       <x:c r="A13" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B13" s="1">
         <x:v>1033275</x:v>
@@ -2894,10 +2894,10 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C2" s="1">
         <x:v>10049014</x:v>
@@ -2905,10 +2905,10 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C3" s="1">
         <x:v>350000</x:v>
@@ -2916,10 +2916,10 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B4" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C4" s="1">
         <x:v>836118</x:v>
@@ -2927,10 +2927,10 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C5" s="1">
         <x:v>2232549</x:v>
@@ -2938,10 +2938,10 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C6" s="1">
         <x:v>650000</x:v>
@@ -2949,10 +2949,10 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="1">
         <x:v>2123261</x:v>
@@ -2960,10 +2960,10 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C8" s="1">
         <x:v>13158948</x:v>
@@ -2971,10 +2971,10 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="1">
         <x:v>1075707</x:v>
@@ -2982,10 +2982,10 @@
     </x:row>
     <x:row r="10" spans="1:3">
       <x:c r="A10" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C10" s="1">
         <x:v>850000</x:v>
@@ -2993,10 +2993,10 @@
     </x:row>
     <x:row r="11" spans="1:3">
       <x:c r="A11" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="1">
         <x:v>600000</x:v>
@@ -3004,10 +3004,10 @@
     </x:row>
     <x:row r="12" spans="1:3">
       <x:c r="A12" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C12" s="1">
         <x:v>91847</x:v>
@@ -3015,10 +3015,10 @@
     </x:row>
     <x:row r="13" spans="1:3">
       <x:c r="A13" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C13" s="1">
         <x:v>161896</x:v>
@@ -3026,10 +3026,10 @@
     </x:row>
     <x:row r="14" spans="1:3">
       <x:c r="A14" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C14" s="1">
         <x:v>350000</x:v>
@@ -3037,10 +3037,10 @@
     </x:row>
     <x:row r="15" spans="1:3">
       <x:c r="A15" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C15" s="1">
         <x:v>2009154</x:v>
@@ -3048,10 +3048,10 @@
     </x:row>
     <x:row r="16" spans="1:3">
       <x:c r="A16" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C16" s="1">
         <x:v>1750000</x:v>
@@ -3059,10 +3059,10 @@
     </x:row>
     <x:row r="17" spans="1:3">
       <x:c r="A17" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C17" s="1">
         <x:v>1564215</x:v>
@@ -3070,10 +3070,10 @@
     </x:row>
     <x:row r="18" spans="1:3">
       <x:c r="A18" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C18" s="1">
         <x:v>1033275</x:v>

</xml_diff>